<commit_message>
auto: 更新 Swing Pattern (US) 2026-09-20
</commit_message>
<xml_diff>
--- a/US_Swing_Pattern.xlsx
+++ b/US_Swing_Pattern.xlsx
@@ -7416,7 +7416,11 @@
       <c r="AH79" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="AI79" s="2" t="inlineStr"/>
+      <c r="AI79" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="AJ79" s="2" t="inlineStr">
         <is>
           <t>柱≥0</t>
@@ -9799,7 +9803,7 @@
         <v>-17.9</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>1.59</v>
+        <v>1.57</v>
       </c>
       <c r="H107" s="2" t="inlineStr"/>
       <c r="I107" s="2" t="inlineStr"/>
@@ -10257,7 +10261,7 @@
       </c>
       <c r="X112" s="2" t="inlineStr"/>
       <c r="Y112" s="2" t="n">
-        <v>-114.63</v>
+        <v>-114.62</v>
       </c>
       <c r="Z112" s="2" t="n">
         <v>-45.78</v>
@@ -11187,7 +11191,7 @@
         <v>-22.8</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>-4.37</v>
+        <v>-4.39</v>
       </c>
       <c r="H123" s="2" t="inlineStr"/>
       <c r="I123" s="2" t="inlineStr"/>
@@ -14429,7 +14433,7 @@
       <c r="W161" s="2" t="inlineStr"/>
       <c r="X161" s="2" t="inlineStr"/>
       <c r="Y161" s="2" t="n">
-        <v>-7.55</v>
+        <v>-7.54</v>
       </c>
       <c r="Z161" s="2" t="n">
         <v>-13.49</v>
@@ -15793,7 +15797,7 @@
         <v>-14.4</v>
       </c>
       <c r="G177" s="2" t="n">
-        <v>9.69</v>
+        <v>9.65</v>
       </c>
       <c r="H177" s="2" t="inlineStr"/>
       <c r="I177" s="2" t="inlineStr"/>
@@ -16561,7 +16565,7 @@
         <v>-0.8</v>
       </c>
       <c r="G186" s="2" t="n">
-        <v>-17.25</v>
+        <v>-17.26</v>
       </c>
       <c r="H186" s="2" t="inlineStr"/>
       <c r="I186" s="2" t="inlineStr"/>
@@ -19027,7 +19031,7 @@
       </c>
       <c r="X215" s="2" t="inlineStr"/>
       <c r="Y215" s="2" t="n">
-        <v>35.39</v>
+        <v>35.4</v>
       </c>
       <c r="Z215" s="2" t="n">
         <v>4.09</v>
@@ -20289,7 +20293,7 @@
         <v>-5.7</v>
       </c>
       <c r="G230" s="2" t="n">
-        <v>-10.97</v>
+        <v>-11</v>
       </c>
       <c r="H230" s="2" t="inlineStr"/>
       <c r="I230" s="2" t="inlineStr"/>
@@ -21085,7 +21089,7 @@
         <v>-7.6</v>
       </c>
       <c r="G239" s="2" t="n">
-        <v>3.97</v>
+        <v>3.96</v>
       </c>
       <c r="H239" s="2" t="inlineStr"/>
       <c r="I239" s="2" t="inlineStr"/>
@@ -22459,7 +22463,7 @@
       <c r="O255" s="2" t="inlineStr"/>
       <c r="P255" s="2" t="inlineStr"/>
       <c r="Q255" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R255" s="2" t="inlineStr"/>
       <c r="S255" s="2" t="inlineStr"/>
@@ -23325,7 +23329,7 @@
         </is>
       </c>
       <c r="C265" s="2" t="n">
-        <v>65.605</v>
+        <v>65.61</v>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
@@ -23365,10 +23369,10 @@
       <c r="W265" s="2" t="inlineStr"/>
       <c r="X265" s="2" t="inlineStr"/>
       <c r="Y265" s="2" t="n">
-        <v>-1.51</v>
+        <v>-1.5</v>
       </c>
       <c r="Z265" s="2" t="n">
-        <v>-11.7</v>
+        <v>-11.69</v>
       </c>
       <c r="AA265" s="2" t="n">
         <v>2.44</v>
@@ -23377,7 +23381,7 @@
         <v>-2.01</v>
       </c>
       <c r="AC265" s="2" t="n">
-        <v>-4.64</v>
+        <v>-4.63</v>
       </c>
       <c r="AD265" s="2" t="n">
         <v>-12.1</v>
@@ -28547,7 +28551,7 @@
         <v>9</v>
       </c>
       <c r="Q325" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R325" s="2" t="inlineStr"/>
       <c r="S325" s="2" t="inlineStr"/>
@@ -28965,7 +28969,7 @@
         <v>-1.2</v>
       </c>
       <c r="G330" s="2" t="n">
-        <v>-1.55</v>
+        <v>-1.43</v>
       </c>
       <c r="H330" s="2" t="inlineStr"/>
       <c r="I330" s="2" t="inlineStr"/>
@@ -29011,7 +29015,7 @@
         <v>56.9</v>
       </c>
       <c r="AE330" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AF330" s="2" t="inlineStr"/>
       <c r="AG330" s="2" t="inlineStr"/>
@@ -30611,25 +30615,25 @@
       <c r="W349" s="2" t="inlineStr"/>
       <c r="X349" s="2" t="inlineStr"/>
       <c r="Y349" s="2" t="n">
-        <v>10.32</v>
+        <v>10.12</v>
       </c>
       <c r="Z349" s="2" t="n">
         <v>-5.26</v>
       </c>
       <c r="AA349" s="2" t="n">
-        <v>1.73</v>
+        <v>1.74</v>
       </c>
       <c r="AB349" s="2" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="AC349" s="2" t="n">
         <v>-3.98</v>
       </c>
       <c r="AD349" s="2" t="n">
-        <v>0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="AE349" s="2" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="AF349" s="2" t="inlineStr"/>
       <c r="AG349" s="2" t="n">
@@ -31407,7 +31411,7 @@
       <c r="W358" s="2" t="inlineStr"/>
       <c r="X358" s="2" t="inlineStr"/>
       <c r="Y358" s="2" t="n">
-        <v>-55.43</v>
+        <v>-55.42</v>
       </c>
       <c r="Z358" s="2" t="n">
         <v>-21.21</v>
@@ -34131,7 +34135,7 @@
       <c r="E390" s="2" t="n"/>
       <c r="F390" s="2" t="n"/>
       <c r="G390" s="2" t="n">
-        <v>103.59</v>
+        <v>103.58</v>
       </c>
       <c r="H390" s="2" t="inlineStr"/>
       <c r="I390" s="2" t="inlineStr"/>
@@ -38007,7 +38011,7 @@
         <v>-7.7</v>
       </c>
       <c r="G435" s="2" t="n">
-        <v>-13.27</v>
+        <v>-13.33</v>
       </c>
       <c r="H435" s="2" t="inlineStr"/>
       <c r="I435" s="2" t="inlineStr"/>
@@ -38050,7 +38054,7 @@
         <v>-8.039999999999999</v>
       </c>
       <c r="AD435" s="2" t="n">
-        <v>-11.7</v>
+        <v>-11.8</v>
       </c>
       <c r="AE435" s="2" t="n">
         <v>13</v>
@@ -44683,7 +44687,7 @@
         <v>0.2</v>
       </c>
       <c r="G515" s="2" t="n">
-        <v>0.75</v>
+        <v>0.67</v>
       </c>
       <c r="H515" s="2" t="inlineStr"/>
       <c r="I515" s="2" t="inlineStr"/>
@@ -45647,7 +45651,7 @@
         <v>-7.7</v>
       </c>
       <c r="G527" s="2" t="n">
-        <v>-8.83</v>
+        <v>-8.869999999999999</v>
       </c>
       <c r="H527" s="2" t="inlineStr"/>
       <c r="I527" s="2" t="inlineStr"/>
@@ -45684,7 +45688,7 @@
         <v>-6.38</v>
       </c>
       <c r="AD527" s="2" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
       <c r="AE527" s="2" t="n">
         <v>20</v>
@@ -45729,7 +45733,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-19 | 526 只</t>
+          <t>截至: 2026-09-20 | 526 只</t>
         </is>
       </c>
     </row>

</xml_diff>